<commit_message>
bue me quedo tremendo cacho de error, dsp lo arreglo
</commit_message>
<xml_diff>
--- a/IA/tablas_generadas/tablita.xlsx
+++ b/IA/tablas_generadas/tablita.xlsx
@@ -436,7 +436,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>PcComponentes</t>
+          <t>Newegg</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -446,12 +446,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Newegg</t>
+          <t>Micro Center</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>PCPartPicker</t>
+          <t>PCity</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -468,25 +468,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Utiliza tipografías Sans-serif claras que garantizan una excelente legibilidad en todas las secciones. El tamaño y espaciado favorecen una lectura cómoda y eficiente.</t>
+          <t>Newegg es conocido por su enfoque limpio. Su tipografía clara y el espaciado adecuado mejoran la legibilidad de descripciones de productos y especificaciones técnicas, facilitando la navegación.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Presenta tipografías estándar y un diseño funcional que prioriza la información. La legibilidad es alta, aunque el volumen de texto puede resultar denso en ocasiones.</t>
+          <t>Amazon utiliza una tipografía sencilla y familiar. La consistencia en el tamaño y estilo de fuente en todo el sitio garantiza una experiencia de lectura cómoda y accesible para los usuarios.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Emplea fuentes limpias y tamaños adecuados para asegurar una lectura fluida. La jerarquía visual de los textos ayuda a identificar rápidamente la información clave.</t>
+          <t>Micro Center presenta una fuente estándar para su contenido. El contraste de colores y la jerarquía visual de su texto ayudan a los usuarios a diferenciar fácilmente la información clave del producto y las ofertas.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>La tipografía es funcional y clara, aunque en ocasiones la uniformidad de tamaño puede dificultar la jerarquía visual de contenidos importantes.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>PCity emplea una tipografía limpia y estándar que asegura una buena legibilidad general. Los títulos son claros, aunque la jerarquía visual entre diferentes elementos de texto podría ser más pronunciada para guiar mejor al usuario.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Se podría mejorar la jerarquía visual del texto y el contraste para destacar información crucial, haciendo que la lectura sea más dinámica y menos monótona.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -496,25 +500,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Su vibrante paleta de colores corporativos (naranja y blanco/gris) es consistente, creando una identidad de marca moderna y fácilmente reconocible en todo el sitio.</t>
+          <t>Newegg emplea una paleta de colores corporativos. Su combinación de azul y blanco se asocia fuertemente con la tecnología, transmitiendo una imagen de fiabilidad y modernidad en el mercado de PC.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Utiliza una paleta de colores simple y reconocible (azul, naranja, blanco). El branding se centra en la familiaridad y confianza, con un logo omnipresente.</t>
+          <t>Amazon se distingue por su distintivo esquema de colores. El negro, naranja y blanco son inmediatamente reconocibles, proyectando una imagen de marca global que es confiable y de fácil acceso.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Predominan los tonos azules y grises, que transmiten profesionalidad y tecnología. El branding es sutil pero consistente, reforzando su imagen en el sector.</t>
+          <t>Micro Center utiliza un esquema de color vibrante en su diseño. La combinación de rojo y negro crea una identidad de marca enérgica, atrayendo a entusiastas de la tecnología con su estilo audaz.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>La interfaz usa colores básicos (azul, blanco, negro) de forma consistente. El branding es funcional, centrado en la herramienta más que en una estética llamativa.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>PCity utiliza un esquema de colores azul y blanco, que es común en tecnología y transmite limpieza. La identidad de marca es funcional, pero podría desarrollarse para ser más distintiva y memorable.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>La identidad de marca podría reforzarse con una paleta de colores más consistente que refleje mejor su propuesta de valor, creando una impresión más cohesionada y memorable.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -524,25 +532,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Destaca por imágenes de producto de alta resolución y vídeos descriptivos. Los iconos son intuitivos y complementan la información textual, mejorando la experiencia de compra.</t>
+          <t>Newegg muestra imágenes de productos de alta calidad y diseños consistentes. La disposición de los elementos visuales es ordenada y profesional, mejorando la experiencia de compra y la presentación de los artículos.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Abundantes imágenes de productos y vistas de 360 grados. Los elementos visuales son informativos y funcionales, aunque el diseño general puede parecer menos moderno.</t>
+          <t>Amazon gestiona una vasta cantidad de elementos visuales con gran eficacia. Desde imágenes de productos hasta banners promocionales, todo está optimizado para cargar rápidamente y ser visualmente atractivo.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ofrece imágenes de productos detalladas y galerías interactivas. Los elementos gráficos son limpios y contribuyen a una presentación profesional del hardware.</t>
+          <t>Micro Center incorpora elementos visuales dinámicos y organizados. Sus banners y gráficos promocionales son efectivos para destacar ofertas, manteniendo una estética limpia que facilita la exploración de productos.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Los elementos visuales son principalmente imágenes de productos, esquemas y gráficos para compatibilidad. Son funcionales, pero la estética es secundaria a la claridad informativa.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>PCity presenta imágenes de productos claras y bien enmarcadas sobre un fondo blanco, lo que contribuye a una apariencia limpia. Se observa una consistencia en el tamaño de las miniaturas, pero faltan elementos gráficos más dinámicos o iconos informativos.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Considerar la inclusión de elementos gráficos más dinámicos y el uso de iconos informativos para mejorar la interacción visual, aportando mayor riqueza sin sobrecargar el diseño.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -552,25 +564,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Navegación intuitiva con menús desplegables claros y un buscador eficiente. La experiencia de usuario es fluida, facilitando la búsqueda y compra de componentes.</t>
+          <t>Newegg ofrece una navegación estructurada y lógica. Sus menús desplegables y filtros avanzados permiten a los usuarios encontrar productos específicos con facilidad, proporcionando una experiencia de usuario eficiente.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>La navegación es amplia y familiar, aunque a veces saturada. La UX se enfoca en la eficiencia del proceso de compra, con un flujo bien establecido y conocido.</t>
+          <t>Amazon es un referente en navegación, con menús intuitivos y una barra de búsqueda potente. La experiencia del usuario es fluida, permitiendo una exploración y compra de productos sin esfuerzo y altamente eficiente.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Presenta una navegación lógica y estructurada, con categorías bien definidas. La UX está diseñada para exploradores de tecnología, con filtros avanzados y fácil acceso a comparativas.</t>
+          <t>Micro Center proporciona una navegación clara y categorizada. Sus opciones de filtro y búsqueda permiten una exploración eficiente del inventario, mejorando la usabilidad para compradores de tecnología.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Navegación clara y orientada a la función, facilitando la búsqueda y compatibilidad de componentes. La UX es altamente funcional, ideal para construir PCs paso a paso.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>PCity ofrece una navegación sencilla con enlaces en el encabezado que son fáciles de entender. La barra de búsqueda es prominente. Sin embargo, se podrían añadir más opciones de filtrado o categorización para una mejor experiencia.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Se podría optimizar la navegación añadiendo filtros más específicos y una categorización más profunda para facilitar la búsqueda de productos, mejorando la experiencia del usuario y la eficiencia.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -580,25 +596,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Contenido bien jerarquizado y organizado por categorías y subcategorías claras. La estructura facilita la exploración y búsqueda de productos específicos.</t>
+          <t>Newegg organiza su contenido de manera lógica y coherente. Las categorías de productos están bien definidas, facilitando que los usuarios exploren y encuentren rápidamente lo que buscan en un catálogo extenso.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Organización de contenido vasta y compleja, pero con una estructura de categorías coherente. Permite una buena visibilidad de productos, a pesar de la enorme oferta.</t>
+          <t>Amazon presenta una estructura de contenido ejemplar. La organización por categorías, recomendaciones y la clara disposición de la información del producto facilitan una interacción intuitiva y eficiente para el usuario.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Estructura lógica y bien definida, optimizada para el hardware. Las fichas de producto son detalladas, y las guías de compra están bien integradas.</t>
+          <t>Micro Center mantiene una organización clara y estructurada. Las secciones de productos y las páginas de categorías están bien definidas, lo que ayuda a los usuarios a navegar sin problemas a través de su amplio inventario.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>La estructura se centra en la compatibilidad de componentes, con listas y filtros. Es muy organizada para su propósito específico de montaje de PCs.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>PCity presenta una estructura organizada con una sección destacada para 'Componentes populares'. El diseño es limpio y los elementos principales están bien posicionados, pero una mayor profundidad en la categorización sería beneficiosa.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Se sugiere una estructura de contenido más jerárquica con categorías y subcategorías más detalladas, lo que permitiría una exploración más profunda y organizada de la oferta de productos.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -608,25 +628,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cumple con estándares básicos de accesibilidad, aunque siempre hay margen de mejora. Se percibe un esfuerzo por hacer el sitio usable para diversos usuarios.</t>
+          <t>Newegg se esfuerza por una buena accesibilidad, usando alto contraste en su texto y un diseño responsive. Se enfoca en garantizar que la información sea legible para una amplia gama de usuarios, mejorando la inclusión.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invierte en accesibilidad para un público global. Presenta opciones para personalizar la experiencia, buscando ser inclusivo para usuarios con diversas necesidades.</t>
+          <t>Amazon es un líder en accesibilidad, con características como descripciones de imágenes y navegación por teclado. Se aseguran de que su plataforma sea utilizable por personas con diversas necesidades, promoviendo la inclusión.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Se esfuerza en ofrecer un sitio accesible, con etiquetas Alt en imágenes y buen contraste. Apunta a la inclusión, aunque no es su característica principal.</t>
+          <t>Micro Center tiene un diseño con buen contraste y tamaños de fuente legibles. La accesibilidad general parece pensada, aunque se podría profundizar en características para usuarios con necesidades especiales.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>La accesibilidad básica está presente en su diseño funcional y textual. Sin embargo, podría beneficiarse de una auditoría WCAG para optimizar la experiencia inclusiva.</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>PCity muestra un buen contraste entre el texto y el fondo, lo cual es positivo para la legibilidad. Los tamaños de fuente son adecuados. Sin embargo, no se observa evidencia de características avanzadas de accesibilidad.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Podría explorar la implementación de funciones de accesibilidad avanzadas, como etiquetas alt para imágenes y navegación por teclado, para asegurar una experiencia inclusiva para todos los usuarios.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -636,25 +660,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ofrece filtros avanzados, comparadores de productos y un configurador de PC muy completo. Estas funcionalidades mejoran significativamente la decisión de compra.</t>
+          <t>Newegg ofrece una funcionalidad robusta, incluyendo búsqueda avanzada, filtrado detallado y comparación de productos. Estas herramientas son esenciales para una experiencia de compra eficiente y satisfactoria en línea.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Funcionalidades robustas, incluyendo el carrito, la lista de deseos y el seguimiento de pedidos. Su proceso de compra es altamente eficiente y consolidado.</t>
+          <t>Amazon es sinónimo de funcionalidad integral, desde la búsqueda de productos hasta el proceso de compra. Ofrece características avanzadas como seguimiento de pedidos y reseñas de usuarios, enriqueciendo la experiencia.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Dispone de herramientas como configuradores de PC, filtros exhaustivos y listas de compatibilidad. Su funcionalidad es clave para usuarios expertos en hardware.</t>
+          <t>Micro Center proporciona funcionalidades sólidas, como filtros de búsqueda detallados y una interfaz de carrito de compras intuitiva. Estas herramientas mejoran la capacidad del usuario para encontrar y adquirir productos.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Su funcionalidad principal es la verificación de compatibilidad de componentes, filtros potentes y guías de montaje. Es esencialmente una herramienta interactiva.</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>PCity parece ofrecer las funcionalidades básicas esperadas, como una barra de búsqueda y visualización de productos. Sin embargo, la imagen no permite evaluar características avanzadas como filtros detallados o una herramienta de comparación de productos.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Sería beneficioso integrar funcionalidades avanzadas como filtros de búsqueda más potentes, herramientas de comparación de productos y un sistema de reseñas para enriquecer la experiencia del usuario.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -664,25 +692,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Incorpora chats en vivo, opiniones de usuarios, y opciones de personalización en configuradores. Fomenta la participación y la toma de decisiones informada.</t>
+          <t>Newegg fomenta la interactividad a través de reseñas de productos, preguntas y respuestas, y configuradores de PC. Estas características permiten a los usuarios participar activamente, mejorando la toma de decisiones de compra.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Alta interactividad a través de reseñas, preguntas y respuestas, y recomendaciones personalizadas. Fomenta un ecosistema de compra y comunidad activo.</t>
+          <t>Amazon potencia la interactividad con un sistema de valoraciones, preguntas y respuestas, y recomendaciones personalizadas. Esto crea una comunidad activa y mejora la relevancia del contenido para cada usuario.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ofrece foros de discusión, comentarios detallados de productos y guías interactivas. Mantiene a los usuarios comprometidos y explorando su catálogo técnico.</t>
+          <t>Micro Center permite la interacción a través de las valoraciones de productos y las secciones de preguntas. Esta interactividad contribuye a la confianza del cliente, ofreciendo una perspectiva comunitaria valiosa.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>La interactividad se centra en la selección de componentes y la visualización de compatibilidades. Podría añadir más elementos sociales o de gamificación para engagement.</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>PCity, por lo que se ve en la imagen, tiene una interactividad limitada a los elementos de navegación. No se observan características como reseñas de usuarios o herramientas de configuración de productos, lo cual es una oportunidad de mejora.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Se sugiere incorporar elementos interactivos como valoraciones y comentarios de usuarios, además de herramientas configurables, para fomentar una mayor participación y generar confianza en la plataforma.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -692,67 +724,91 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Goza de una excelente visibilidad en buscadores, con una estrategia SEO bien definida y un contenido optimizado para el mercado de PC en español.</t>
+          <t>Newegg optimiza su sitio para SEO, utilizando descripciones detalladas, palabras clave relevantes y una estructura de URL amigable. Esto asegura una alta visibilidad en los motores de búsqueda, atrayendo a más usuarios.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Domina el SEO por su autoridad de dominio y la vasta cantidad de contenido. Su visibilidad es inigualable en un amplio espectro de búsquedas de productos.</t>
+          <t>Amazon tiene una estrategia de SEO robusta, capitalizando su autoridad de dominio y optimizando las páginas de productos. Esto garantiza que sus vastos listados sean fácilmente descubiertos por los usuarios que buscan productos específicos.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Presenta un SEO sólido, especialmente para búsquedas de hardware específico. Su contenido técnico y la estructura del sitio favorecen un buen posicionamiento.</t>
+          <t>Micro Center utiliza descripciones de productos optimizadas y categorías claras para SEO. Esto les permite clasificar bien para términos de búsqueda relevantes, atrayendo tráfico orgánico interesado en hardware.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Su SEO es bueno para búsquedas específicas de compatibilidad y construcción de PCs. La optimización de palabras clave podría enfocarse en guías y tutoriales para mejorar aún más.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>Aunque no se puede evaluar directamente desde la imagen, un buen SEO es crucial. La estructura de URL y las descripciones de los productos serían puntos clave de optimización para mejorar la visibilidad orgánica.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Para mejorar la visibilidad orgánica, se recomienda optimizar la estructura de las URL, implementar meta descripciones y títulos atractivos, y asegurar que el contenido esté enriquecido con palabras clave relevantes.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Performance/Loading Speed</t>
+          <t>Performance &amp; Loading Speed</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mantiene una velocidad de carga rápida y un rendimiento optimizado. Esto asegura una experiencia de navegación fluida y satisfactoria para el usuario.</t>
+          <t>Newegg optimiza continuamente su rendimiento. Sus páginas cargan rápidamente, incluso con gran cantidad de contenido, lo que es crucial para retener a los usuarios y mejorar la experiencia de compra en línea.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A pesar de su enorme complejidad, Amazon carga relativamente rápido. Su rendimiento está altamente optimizado para manejar un volumen masivo de tráfico y productos.</t>
+          <t>Amazon invierte fuertemente en la velocidad de carga de su sitio. Esto garantiza una experiencia de usuario fluida, reduciendo la tasa de rebote y mejorando la satisfacción general del cliente, incluso con contenido masivo.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ofrece una buena velocidad de carga y un rendimiento web estable. La optimización de imágenes y scripts contribuye a una experiencia ágil.</t>
+          <t>Micro Center tiene un rendimiento decente, con tiempos de carga de página aceptables. Mantener una velocidad de carga rápida es vital para la satisfacción del usuario y las clasificaciones de los motores de búsqueda.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>La velocidad de carga es eficiente, dado el volumen de datos de compatibilidad que maneja. La optimización continua de recursos es clave para mantener la fluidez.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>Sin datos de prueba, la velocidad de carga no es visible. Sin embargo, un diseño limpio y pocas animaciones pueden contribuir a un rendimiento rápido, fundamental para la retención de usuarios y el SEO.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Asegurar que el sitio web cargue rápidamente es primordial; se debería optimizar imágenes, usar caché y minificar recursos para una experiencia fluida, especialmente en dispositivos móviles.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>+Final Conclusion</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+          <t>Final Conclusion</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Newegg es un referente en e-commerce de hardware. Su sólida interfaz, extenso catálogo y servicio al cliente lo posicionan como una opción preferente para entusiastas y profesionales de la tecnología, destacando en todos los criterios.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Amazon es un gigante del comercio electrónico. Su escala, conveniencia y experiencia de usuario optimizada, respaldadas por un robusto sistema logístico, lo convierten en una plataforma dominante y globalmente accesible para cualquier compra.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Micro Center sobresale en la venta minorista de componentes. Su combinación de presencia en línea y tiendas físicas, junto con un enfoque en el servicio experto, ofrece una experiencia de compra completa y especializada.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PCity presenta una base prometedora con un diseño limpio y navegación directa. Sus elementos visuales son claros, ofreciendo una experiencia básica pero funcional para el usuario. La usabilidad es notable, aunque sin lujos. Se enfoca en la simplicidad.</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>El sitio web analizado posee una base sólida en su estructura y funcionalidades esenciales, ofreciendo una experiencia adecuada para el usuario. Sin embargo, para capitalizar su potencial, se sugiere optimizar la jerarquía visual y la interactividad. Mejorar el rendimiento de carga e implementar una estrategia SEO más robusta también potenciarían su visibilidad y engagement. Se recomienda explorar nuevas funcionalidades para enriquecer la oferta y destacarse en el competitivo mercado.</t>
+          <t>En general, el sitio presenta un diseño limpio y una navegación intuitiva, lo que son puntos fuertes. Las principales oportunidades de mejora residen en enriquecer la interactividad y la funcionalidad avanzada, así como en profundizar la estructura del contenido para ofrecer una experiencia más completa y distintiva a los usuarios.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
la rompi wacho. ya te genera el codigo todo piola
</commit_message>
<xml_diff>
--- a/IA/tablas_generadas/tablita.xlsx
+++ b/IA/tablas_generadas/tablita.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:AT12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,25 +436,225 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Tom's Hardware</t>
+          <t>Newegg.com: Se observa una tipografía clara y bien contrastada. El texto es fácilmente legible, con tamaños adecuados para el contenido principal y secundario.</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Newegg</t>
+          <t>PcComponentes.com: Presenta una combinación de fuentes que favorece la legibilidad. La jerarquía visual del texto está bien definida, mejorando la experiencia de lectura.</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>GamersNexus</t>
+          <t>Amazon.com (Sección de Componentes PC): Emplea fuentes estándar que aseguran una alta legibilidad en diversos dispositivos. La densidad del texto se gestiona para evitar la sobrecarga visual.</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Pcity</t>
+          <t>Sitio Web de la Imagen: La selección tipográfica parece moderna y funcional. La claridad del texto es un punto fuerte, aunque el espaciado en algunos bloques podría optimizarse.</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg.com: Utiliza una paleta de colores distintiva que refuerza su identidad. Los tonos fríos predominan, aportando una sensación de tecnología y profesionalismo.</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PcComponentes.com: Su identidad de marca se transmite eficazmente a través de una paleta vibrante. Los colores se usan estratégicamente para destacar promociones y áreas clave.</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon.com (Sección de Componentes PC): Los colores reflejan una marca reconocida globalmente, con un uso consistente en elementos clave. La neutralidad del fondo permite que los productos resalten fácilmente.</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sitio Web de la Imagen: La paleta de colores es coherente con el sector tecnológico. La marca se expresa con tonos modernos y un logotipo bien integrado, aunque podría explorar más dinamismo en las llamadas a la acción.</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg.com: Las imágenes de productos son de alta calidad y se complementan con gráficos informativos. Los iconos son intuitivos, facilitando la comprensión rápida del contenido.</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>PcComponentes.com: Incorpora elementos visuales atractivos y bien organizados. Las animaciones y los banners promocionales son impactantes sin distraer la navegación principal.</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon.com (Sección de Componentes PC): Destaca por la gran cantidad de imágenes y vídeos de productos. La organización visual es crucial para manejar el vasto catálogo, utilizando miniaturas claras.</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Sitio Web de la Imagen: Las imágenes de productos son nítidas y detalladas, con una buena integración en el diseño. Se usan gráficos claros, pero la variedad en los tipos de visuales podría ampliarse.</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg.com: Ofrece una navegación intuitiva y eficiente, con menús bien estructurados. La experiencia de usuario se optimiza con filtros avanzados y una búsqueda robusta.</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>PcComponentes.com: La estructura de navegación es clara, permitiendo a los usuarios encontrar productos fácilmente. El flujo de compra se diseña para ser directo y sin fricciones.</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon.com (Sección de Componentes PC): La navegación es excepcionalmente funcional para un catálogo tan extenso. La experiencia de usuario se ve reforzada por un sistema de categorías y subcategorías detallado.</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Sitio Web de la Imagen: La navegación es lógica y los menús son accesibles. La experiencia del usuario es en general positiva, aunque el proceso de filtrado podría ser más prominente o intuitivo.</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg.com: El contenido está lógicamente organizado en categorías claras. Las páginas de productos presentan una estructura uniforme, facilitando la comparación y la toma de decisiones.</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>PcComponentes.com: La estructura del sitio es muy organizada, lo que facilita la exploración de productos. Las secciones están bien delimitadas, proporcionando un acceso rápido a la información relevante.</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon.com (Sección de Componentes PC): Pese a su tamaño, mantiene una organización coherente y estructurada. La disposición de la información en las páginas de resultados y productos es predecible y sencilla.</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Sitio Web de la Imagen: La estructura general del sitio es coherente y fácil de seguir. La organización de las categorías de productos es clara, aunque la disposición de algunos elementos en la página de inicio podría ser más dinámica.</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg.com: Se esfuerza por ser accesible, aunque puede haber áreas de mejora en contraste. La compatibilidad con tecnologías de asistencia podría ser revisada para una mayor inclusión.</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>PcComponentes.com: Implementa características básicas de accesibilidad, como texto alternativo en imágenes. Se observa un esfuerzo por cumplir con estándares, pero hay margen para optimizaciones adicionales.</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon.com (Sección de Componentes PC): Considera la accesibilidad con opciones de visualización y navegación claras. La compatibilidad con diversos dispositivos y navegadores es un punto fuerte del diseño universal.</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Sitio Web de la Imagen: El sitio cumple con aspectos básicos de accesibilidad, como contraste de texto. Podría mejorar la navegación para usuarios con discapacidades visuales o motoras.</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg.com: Todas las funciones del sitio, desde la búsqueda hasta el carrito, operan sin fallos. La interactividad de los filtros y las opciones de personalización es fluida.</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>PcComponentes.com: El sitio web es totalmente funcional, con un proceso de compra robusto y eficiente. Las herramientas de configuración de PC funcionan de manera precisa.</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon.com (Sección de Componentes PC): La funcionalidad del sitio es impecable, con un sistema de búsqueda potente y un carrito de compras fiable. Todas las características operan como se espera, brindando confianza al usuario.</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Sitio Web de la Imagen: La funcionalidad es sólida, con todas las herramientas de compra y navegación operativas. Los formularios funcionan correctamente, pero la velocidad de carga en algunas secciones podría ser optimizada.</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg.com: Ofrece diversas opciones de interacción, como comentarios y comparativas de productos. Los elementos interactivos están bien diseñados y responden de forma intuitiva.</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>PcComponentes.com: Fomenta la interacción mediante reseñas de usuarios y un configurador de PCs. Los elementos interactivos están bien implementados, enriqueciendo la experiencia del comprador.</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon.com (Sección de Componentes PC): Proporciona múltiples formas de interactuar, desde valoraciones hasta preguntas y respuestas. La experiencia interactiva está muy pulida, animando a la participación de la comunidad.</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Sitio Web de la Imagen: El sitio permite la interacción a través de reseñas de productos. Podría integrar más herramientas interactivas, como un chat en vivo o configuradores visuales, para enriquecer la experiencia.</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg.com: El sitio utiliza URL amigables y metadescripciones optimizadas. El contenido está estructurado para ser fácilmente rastreable por los motores de búsqueda.</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>PcComponentes.com: Las páginas están optimizadas con palabras clave relevantes y una estructura clara. Esto contribuye a un buen posicionamiento en los resultados de búsqueda.</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon.com (Sección de Componentes PC): Demuestra una fuerte estrategia SEO con un gran volumen de contenido indexable. La autoridad de dominio es alta, lo que beneficia su visibilidad en búsquedas generales.</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Sitio Web de la Imagen: El sitio parece seguir prácticas básicas de SEO, con títulos y descripciones. La optimización de contenido para palabras clave específicas podría ser más agresiva.</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg.com: Mantiene una excelente velocidad de carga en la mayoría de sus páginas. La optimización de imágenes y scripts contribuye a un rendimiento general sobresaliente.</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>PcComponentes.com: Ofrece un rendimiento rápido y constante, incluso con elementos multimedia. La optimización del servidor y el almacenamiento en caché contribuyen a una navegación fluida.</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon.com (Sección de Componentes PC): Su infraestructura permite una carga rápida, a pesar de la complejidad del sitio. La experiencia del usuario se beneficia de la minimización de tiempos de espera en todas las secciones.</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Sitio Web de la Imagen: La velocidad de carga es aceptable en general, pero algunas páginas cargan más lento. La optimización de recursos y la implementación de técnicas de caché podrían mejorar esto.</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Newegg.com: </t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PcComponentes.com: </t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amazon.com (Sección de Componentes PC): </t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sitio Web de la Imagen: </t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>conclusion</t>
         </is>
@@ -466,29 +666,53 @@
           <t>Typography &amp; Readability</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Presenta un estilo tipográfico claro y profesional. Facilita la lectura de artículos extensos con buen contraste y tamaño de fuente, optimizando la experiencia de usuario.</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Utiliza fuentes estándar de e-commerce, con buena legibilidad en listados de productos. La densidad de información podría beneficiarse de un enfoque más organizado, mejorando la claridad.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Exhibe una tipografía técnica y directa. Proporciona una experiencia de lectura enfocada en el detalle, ideal para usuarios que buscan información muy específica sobre hardware.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Emplea tipografía sencilla y legible. El texto principal es claro, pero la consistencia y jerarquía en diversas secciones podrían optimizarse para una mejor comprensión visual del contenido.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>The site in the image uses clear fonts for main headings and product names, but body text consistency and hierarchical sizing could enhance information consumption across various screen sizes.</t>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>Para mejorar, este sitio podría ajustar el espaciado entre líneas en ciertos elementos de texto. Mantener la legibilidad actual es crucial, y una revisión de la consistencia en estilos de párrafo sería beneficiosa.</t>
         </is>
       </c>
     </row>
@@ -498,29 +722,53 @@
           <t>Colors &amp; Branding</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Mantiene una paleta de colores sobria y tecnológica. Su branding global es consistente, transmitiendo autoridad y fiabilidad en el ámbito de la tecnología.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Adopta una combinación de colores vibrante y comercial. El branding minorista es reconocible, con un enfoque claro en ofertas y categorías de productos destacadas.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Usa una estética oscura enfocada en el rendimiento. El branding es distintivo en su nicho, reflejando contenido técnico y análisis de hardware sin concesiones.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Presenta una combinación de azul brillante y blanco. El logo y esquema de color sugieren un enfoque moderno y accesible, aunque el branding general podría ser más sofisticado.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>The color scheme is functional and distinctive, but expanding the brand identity beyond the basic blue and white, perhaps with secondary accent colors or graphic elements, could create a more memorable and unique user experience.</t>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>Para evolucionar, el sitio podría introducir acentos de color más audaces para elementos interactivos. Esto impulsaría la participación del usuario y fortalecería el reconocimiento de sus puntos focales.</t>
         </is>
       </c>
     </row>
@@ -530,29 +778,53 @@
           <t>Visual Elements</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Integra imágenes de alta calidad y gráficos informativos. Ofrece visuales pertinentes que complementan eficazmente sus extensas reseñas y análisis técnicos detallados.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Destaca por fotografías de productos claras y detalladas. Las imágenes cumplen su función de mostrar artículos, pero gráficos adicionales son limitados en su presentación general.</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Incorpora imágenes de hardware detalladas y capturas de pantalla de benchmarks. Los elementos visuales son cruciales para sus análisis, apoyando la información técnica con evidencia gráfica.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Muestra imágenes de productos consistentes y bien alineadas. Las miniaturas de componentes populares son claras, pero la inclusión de gráficos o íconos adicionales realzaría la experiencia.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Product images are uniformly presented, which is a good starting point. However, incorporating more diverse visual elements such as infographics, comparison charts, or detailed product galleries could significantly improve user engagement and information retention.</t>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>El sitio podría beneficiarse de la adición de más elementos visuales interactivos. Implementar vídeos cortos de productos o vistas 360 grados mejoraría significativamente la experiencia de usuario y la decisión de compra.</t>
         </is>
       </c>
     </row>
@@ -562,29 +834,53 @@
           <t>Navigation &amp; UX</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Ofrece navegación estructurada y lógica. La experiencia de usuario es intuitiva, permitiendo acceso rápido a categorías de productos, noticias y guías relevantes.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Proporciona navegación robusta orientada al comercio. La experiencia de usuario se centra en búsqueda y filtrado de productos, diseñada para facilitar transacciones eficientes.</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Cuenta con navegación directa a sus categorías de contenido principal. La UX está diseñada para exploradores técnicos, priorizando el acceso a sus profundos análisis y videos.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Tiene una barra de navegación superior clara con enlaces esenciales. La experiencia de usuario parece sencilla, aunque opciones de filtrado o categorías secundarias no son visibles.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>The main navigation is clear and concise, offering immediate access to key sections. To enhance user experience, implementing more dynamic filters, detailed category breakdowns, and a consistent breadcrumb trail would be beneficial for deeper exploration.</t>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>Mejorar la visibilidad y usabilidad de los filtros de búsqueda es una prioridad. Un sistema de filtrado más avanzado y fácilmente perceptible ayudaría a los usuarios a refinar sus elecciones con mayor rapidez y eficiencia.</t>
         </is>
       </c>
     </row>
@@ -594,29 +890,53 @@
           <t>Organization &amp; Structure</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Organiza su contenido en secciones bien definidas. La estructura facilita la búsqueda de información específica, categorizando artículos por tipo de componente y temática tecnológica.</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Presenta organización de productos por categorías lógicas. La estructura está optimizada para la compra, con listados claros y opciones de clasificación para la elección del cliente.</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Estructura su contenido por tipos de análisis y publicaciones. La organización es coherente con su enfoque en rendimiento de hardware, permitiendo encontrar rápidamente estudios detallados.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Muestra componentes populares en un diseño de cuadrícula ordenado. La organización es limpia y funcional, pero no se aprecian categorías avanzadas o árboles de productos.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>The current layout for popular components is clean and easy to scan. Expanding this structure to include clear hierarchical categories, advanced sorting options, and dedicated landing pages for different component types would greatly improve overall site navigability.</t>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>Reorganizar ligeramente la página de inicio para destacar ofertas y novedades. Esto crearía un punto de entrada más atractivo y mantendría a los usuarios interesados en explorar el contenido actual.</t>
         </is>
       </c>
     </row>
@@ -626,29 +946,53 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Se esfuerza por buena accesibilidad en su contenido. Utiliza atributos ALT en imágenes y estructura HTML semántica, aunque siempre hay margen para mejoras.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Implementa características básicas de accesibilidad para su plataforma. Se enfoca en cumplir estándares para facilitar navegación y compra a un amplio rango de usuarios.</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Prioriza la claridad del contenido. La accesibilidad es razonable, pero la complejidad técnica de algunos gráficos podría ser un desafío para usuarios con ciertas discapacidades.</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Parece tener contraste de color adecuado para el texto principal. La disposición simple sugiere una accesibilidad básica, pero se necesita una evaluación completa.</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>The high contrast between blue and white is a positive step for visual accessibility. Further improvements should focus on providing alternative text for all images, ensuring keyboard navigation, and implementing ARIA labels for interactive elements to support screen reader users.</t>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>Priorizar la implementación de una navegación más amigable para teclado. Asegurar que todos los elementos interactivos sean accesibles sin el uso del ratón abrirá el sitio a una audiencia más amplia y diversa.</t>
         </is>
       </c>
     </row>
@@ -658,29 +1002,53 @@
           <t>Functionality</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Ofrece funcionalidad robusta para publicación de contenido. Incluye búsqueda avanzada, comentarios y una base de datos extensa de especificaciones de componentes.</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Dispone de funcionalidad completa de comercio electrónico. Permite búsqueda de productos, gestión de carritos, procesamiento de pagos y seguimiento de pedidos, con experiencia fluida.</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Proporciona funcionalidad para entrega de contenido multimedia. Integra videos y artículos, con herramientas para compartir y comentar, facilitando el engagement con su audiencia.</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Presenta un buscador visible y enlaces a secciones clave. La función 'Arma tu PC' sugiere un configurador, indicando funcionalidad orientada a la utilidad del usuario.</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>The presence of a search bar and a 'Build your PC' section indicates a focus on practical functionality. Enhancements could include advanced comparison tools, a more robust component compatibility checker within the builder, and real-time stock updates for parts.</t>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>Optimizar la velocidad de carga de las páginas de productos es esencial. Un rendimiento más rápido reducirá la tasa de rebote y mejorará la percepción general de eficiencia y modernidad del sitio.</t>
         </is>
       </c>
     </row>
@@ -690,29 +1058,53 @@
           <t>Interactivity</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Permite comentarios en artículos y foros activos. Ofrece oportunidades de interacción para los usuarios, fomentando discusiones y el intercambio de conocimientos sobre tecnología.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Habilita reseñas de productos, preguntas y respuestas de usuarios. La interacción se centra en la comunidad de compradores, facilitando decisiones informadas y el soporte entre pares.</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Fomenta la interacción a través de comentarios en videos y artículos. La comunidad es activa, participando en debates técnicos, enriqueciendo el contenido con perspectivas adicionales.</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>La imagen no muestra elementos interactivos más allá de navegación básica. Secciones como 'Arma tu PC' o 'Comparar' podrían ofrecer interfaces más dinámicas para el usuario.</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>While basic navigation is present, the site could significantly benefit from more interactive elements. Implementing user ratings, a comment section, forums, or a more engaging 'Build your PC' wizard would foster a stronger community and user engagement.</t>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>La integración de un chat en vivo para soporte inmediato sería un gran añadido. Esto proporcionaría asistencia en tiempo real, resolviendo dudas rápidamente y mejorando la satisfacción del cliente.</t>
         </is>
       </c>
     </row>
@@ -722,77 +1114,165 @@
           <t>SEO</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Aplica estrategias SEO sólidas para su vasto contenido. Su alta autoridad de dominio le permite posicionarse bien en búsquedas relacionadas con hardware y tecnología.</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Maneja un SEO robusto enfocado en productos y categorías. Su optimización es clave para captar tráfico de búsqueda transaccional con descripciones y metadatos efectivos.</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Optimiza su contenido para búsquedas de nicho y términos técnicos. Su SEO se centra en rendimiento y análisis detallados, atrayendo audiencia especializada en hardware para PC.</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>La estructura de títulos y claridad del contenido son positivos para el SEO básico. La optimización de metadescripciones, encabezados y URLs amigables es crucial para visibilidad.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>The clear title and content visible suggest a good foundation for SEO. To improve organic reach, a focused strategy including keyword-rich content, optimized meta descriptions, structured data, and a robust internal linking structure should be developed.</t>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>Desarrollar una estrategia de contenido SEO más robusta es vital. Crear guías de compra, comparativas y artículos de blog con palabras clave relevantes atraerá más tráfico orgánico y establecerá el sitio como una autoridad.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Customer Support &amp; Community</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Ofrece foros comunitarios activos y guías extensas. El soporte se centra en autoayuda a través de una rica base de conocimientos generada por expertos y usuarios.</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Proporciona soporte al cliente integral y herramientas de comunidad. Incluye chat en vivo, RMA, FAQs y foros, facilitando una experiencia de compra asistida.</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>No tiene soporte al cliente tradicional, pero sí una comunidad. Sus videos y artículos sirven como apoyo indirecto, respondiendo preguntas comunes a través del contenido.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>La imagen no revela información sobre soporte o comunidad explícita. La sección 'Información' podría albergar FAQs o enlaces de contacto para consultas de usuarios.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>The current layout doesn't explicitly display customer support or community features. Incorporating a dedicated help center, live chat, or a user forum would significantly boost user confidence and provide valuable resources for building or comparing PCs.</t>
+          <t>Performance y Velocidad de Carga</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>Es fundamental invertir en la optimización de recursos, especialmente imágenes y scripts. Implementar Lazy Loading y mejorar el caché del navegador resultaría en una experiencia mucho más fluida.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Final Conclusion</t>
+          <t>Final Conclusion row</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>El sitio de la imagen posee una base sólida con una interfaz limpia y una propuesta de valor clara para construir y comparar PCs. Para mejorar, debería expandir la interactividad con herramientas de configuración más robustas, optimizar la organización del contenido con categorías detalladas, y desarrollar una estrategia SEO y de comunidad más profunda. Se recomienda integrar más elementos visuales informativos y asegurar una accesibilidad completa para todos los usuarios.</t>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>En general, el sitio de la imagen presenta una base sólida con buena legibilidad y funcionalidad. Sin embargo, hay un gran potencial para enriquecer la experiencia del usuario y aumentar la visibilidad. Sugiero enfocarse en elementos interactivos como un chat en vivo y un configurador de productos, mejorar la velocidad de carga de las páginas de detalles, optimizar la usabilidad de los filtros, y robustecer la estrategia de contenido SEO. Estas mejoras no solo atraerán a más usuarios, sino que también los mantendrán comprometidos, fortaleciendo la percepción de su marca en el mercado.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
falta seguir arreglando errores
</commit_message>
<xml_diff>
--- a/IA/tablas_generadas/tablita.xlsx
+++ b/IA/tablas_generadas/tablita.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:AT12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,25 +436,225 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Tom's Hardware</t>
+          <t>Newegg - Emplea una tipografía clara y moderna para los listados de productos. Facilita la lectura de especificaciones detalladas.</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>PC Part Picker</t>
+          <t>Amazon - Utiliza fuentes limpias y tamaños ajustables para diversos contenidos. Mantiene una alta legibilidad en descripciones y reseñas.</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Newegg</t>
+          <t>Micro Center - Presenta textos con una fuente sans-serif estándar que asegura la claridad. La información de los productos es fácil de escanear y comprender.</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>PCity</t>
+          <t>B&amp;H Photo Video - Se observan fuentes nítidas y consistentes en todo el portal. La lectura de las fichas técnicas resulta cómoda y fluida.</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg - La marca se distingue por una paleta de colores vibrantes con acentos rojos y azules. Refleja una imagen de tecnología y dinamismo.</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon - La identidad visual se basa en tonos azules y blancos, que transmiten confianza y seriedad. El logo es reconocido globalmente por su simplicidad.</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Micro Center - Una combinación de colores sobrios y detalles en verde esmeralda define su estética. El diseño general es profesional y enfocado al hardware.</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H Photo Video - La marca emplea una paleta de colores azul y blanco, con toques de naranja para llamadas a la acción. El branding proyecta una imagen de fiabilidad y experiencia.</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg - Se caracteriza por imágenes de alta resolución de productos desde múltiples ángulos. Los videos y configuradores 3D enriquecen la experiencia visual.</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon - Presenta una gran variedad de imágenes de producto, a menudo con zooms detallados. Las infografías y comparativas son frecuentes en sus páginas.</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Micro Center - Destaca por las fotografías de calidad profesional de componentes y sistemas. Los gráficos ilustrativos ayudan a comprender características técnicas.</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H Photo Video - Ofrece fotografías de producto impecables y claras, acompañadas de miniaturas bien organizadas. Los elementos gráficos son limpios y funcionales, aunque no abundan los videos.</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg - Dispone de menús de categorías detallados y un potente motor de búsqueda con filtros avanzados. La experiencia del usuario es eficiente para encontrar productos específicos.</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon - La navegación es intuitiva gracias a un diseño familiar y una barra de búsqueda prominente. El proceso de compra está optimizado para la sencillez.</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Micro Center - Ofrece un sistema de navegación claro con categorías bien definidas y filtros eficaces. La experiencia de usuario es directa y centrada en la búsqueda de hardware.</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H Photo Video - La navegación es lógica y estructurada, con un menú principal bien organizado y una búsqueda efectiva. Los usuarios pueden encontrar rápidamente lo que buscan sin confusión.</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg - El contenido está organizado de manera lógica con secciones claras para productos, guías y ofertas. La arquitectura de la información es profunda pero accesible.</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon - La estructura del contenido es amplia, categorizando millones de productos de forma eficaz. Las páginas de producto están bien segmentadas con toda la información relevante.</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Micro Center - Presenta una estructura de sitio bien definida, separando claramente productos, servicios y recursos. La jerarquía de la información es fácil de seguir.</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H Photo Video - La disposición de los elementos es ordenada y coherente, con categorías de producto claramente definidas y submenús intuitivos. La información se presenta de forma concisa y bien distribuida.</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg - Se esfuerza por ofrecer opciones de accesibilidad, como compatibilidad con lectores de pantalla. Permite a un público amplio interactuar con el contenido.</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon - Incorpora características de accesibilidad como descripciones de imágenes y navegación por teclado. Se mantiene un compromiso para ser inclusivo con todos los usuarios.</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Micro Center - Considera la accesibilidad básica en su diseño web. Busca garantizar que la información esencial sea accesible para la mayoría de los usuarios.</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H Photo Video - El diseño web cumple con estándares básicos de accesibilidad, aunque hay margen para mejoras en contraste y navegación asistida. La experiencia para usuarios con necesidades especiales es funcional.</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg - Proporciona herramientas robustas como creadores de PC personalizados y comparadores de productos. La funcionalidad del carrito de compras es fluida y segura.</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon - Ofrece una funcionalidad completa que incluye seguimiento de pedidos, listas de deseos y múltiples opciones de pago. La plataforma soporta un vasto ecosistema de servicios.</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Micro Center - Incluye funciones clave como constructores de PC, filtros de búsqueda avanzados y soporte en línea. La experiencia de compra es directa y sin complicaciones.</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H Photo Video - Las características funcionales son sólidas, con un carrito de compras eficiente y un sistema de gestión de cuentas completo. La búsqueda por filtros funciona de manera fiable y rápida.</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg - Fomenta la interacción a través de reseñas de usuarios, foros y soporte en vivo. Los elementos interactivos mejoran la toma de decisiones del comprador.</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon - Permite la interacción mediante reseñas de productos, preguntas y respuestas, y recomendaciones personalizadas. Fomenta una comunidad activa de compradores.</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Micro Center - Ofrece algunas características interactivas como reseñas de clientes y un chat de soporte. Busca facilitar la comunicación y resolución de dudas.</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H Photo Video - La interacción se centra en las reseñas de productos, el soporte al cliente y las opciones de personalización de cuenta. Podría beneficiarse de más elementos dinámicos.</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg - Está optimizado para motores de búsqueda con una buena estructura de URLs y contenido relevante. Ocupa posiciones destacadas para términos relacionados con componentes de PC.</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon - Posee una estrategia de SEO robusta, capitalizando su autoridad de dominio para clasificar alto en diversas búsquedas. Su contenido está bien indexado.</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Micro Center - Mantiene una presencia sólida en los resultados de búsqueda para términos de hardware. La optimización SEO permite que los usuarios encuentren fácilmente sus productos.</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H Photo Video - La optimización para motores de búsqueda es efectiva, con una buena indexación de productos y metadatos relevantes. Se clasifica bien para términos específicos de fotografía y video.</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Newegg - Exhibe una velocidad de carga rápida, optimizando la experiencia del usuario. La eficiencia en la entrega de contenido es un pilar fundamental.</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon - Muestra tiempos de carga generalmente eficientes, a pesar de la gran cantidad de contenido. Las imágenes y scripts están bien optimizados.</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Micro Center - Ofrece un buen rendimiento y velocidad de carga para la mayoría de sus páginas. La experiencia es fluida para los usuarios al navegar por el inventario.</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H Photo Video - La plataforma carga de manera consistente y rápida en la mayoría de los dispositivos, garantizando una experiencia de usuario fluida. Los recursos están bien optimizados para la entrega veloz del contenido.</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Newegg - </t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amazon - </t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Micro Center - </t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B&amp;H Photo Video - </t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>conclusion</t>
         </is>
@@ -471,6 +671,46 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -483,6 +723,46 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -495,6 +775,46 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -507,6 +827,46 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -519,6 +879,46 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -531,6 +931,46 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -543,6 +983,46 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -555,6 +1035,46 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -567,11 +1087,51 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Performance &amp; Loading Speed</t>
+          <t>Rendimiento y Velocidad de Carga</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -579,6 +1139,46 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -590,9 +1190,49 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>La plataforma destaca por su clara presentación visual de componentes y una navegación intuitiva. Potenciales mejoras incluyen refinar la coherencia de la tipografía y expandir las opciones de personalización para el usuario.</t>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>El sitio web analizado destaca por su navegación intuitiva y la alta calidad de sus imágenes de producto, facilitando una experiencia de usuario clara y funcional. Sin embargo, podría mejorar en la integración de más elementos interactivos y en la ampliación de sus características de accesibilidad para un público más diverso. Potenciar el uso de videos explicativos y comparativas directas con la competencia fortalecería su propuesta de valor.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
3 horas de trabajo sirvieron para algo 💢
</commit_message>
<xml_diff>
--- a/IA/tablas_generadas/tablita.xlsx
+++ b/IA/tablas_generadas/tablita.xlsx
@@ -436,22 +436,22 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>PcComponentes</t>
+          <t>PcComponentes.com</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Noticias3D</t>
+          <t>Hard Zone</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Profesional Review</t>
+          <t>El Chapuzas Informático</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>(NombrePágina4)</t>
+          <t>Pity PC</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -466,13 +466,29 @@
           <t>Typography &amp; Readability</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Presenta fuentes sans-serif claras y legibles, garantizando una experiencia de lectura fluida para las descripciones de productos.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Utiliza una combinación de tamaños y estilos de fuente que mejoran la jerarquía visual de sus extensos artículos técnicos.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Se beneficia de una tipografía bien espaciada y contrastada, haciendo que el contenido del blog sea muy fácil de digerir.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Los elementos textuales son nítidos y directos, presentando una jerarquía limpia que facilita la comprensión del contenido general.</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Se beneficia de mantener la consistencia en el tamaño de fuente. Destaca por su claridad, pero podría mejorar la jerarquía visual del texto en la página.</t>
+          <t>Considerar la implementación de una mayor variedad de pesos y tamaños de fuente para los encabezados podría mejorar la jerarquía visual. Ajustar el color del texto para un contraste ligeramente más alto podría beneficiar a usuarios con ciertas deficiencias visuales.</t>
         </is>
       </c>
     </row>
@@ -482,13 +498,29 @@
           <t>Colors &amp; Branding</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Su paleta de colores naranja y gris transmite profesionalidad, estableciendo una identidad de marca coherente y reconocible.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>El esquema oscuro con acentos brillantes es distintivo, alineándose perfectamente con su enfoque en el gaming y hardware de alto rendimiento.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Una combinación de azules y blancos domina, proyectando una imagen de seriedad y fiabilidad en su contenido técnico especializado.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Predomina un azul brillante combinado con blanco, otorgando una sensación de energía y frescura. El esquema de color es sencillo y directo.</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>La fuerte identidad visual es un punto positivo. Considerar añadir un color secundario de acento para secciones importantes y reforzar el branding.</t>
+          <t>Aunque el azul crea una identidad fuerte, explorar tonos complementarios podría añadir sofisticación. Introducir colores de acento secundarios podría resaltar mejor los llamados a la acción, mejorando la interacción del usuario.</t>
         </is>
       </c>
     </row>
@@ -498,13 +530,29 @@
           <t>Visual Elements</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Presenta imágenes de productos de alta resolución y gráficos detallados, esenciales para las decisiones de compra informadas.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Incorpora visuales atractivos, incluyendo fotos detalladas e infografías, que enriquecen los artículos técnicos complejos.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Muestra fotografía de producto nítida y gráficos personalizados, elevando el atractivo visual de sus exhaustivas revisiones.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Las imágenes de productos son claras y están bien expuestas en la página principal, lo cual es fundamental para el compromiso visual. La consistencia en el estilo contribuye a una experiencia unificada.</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>La clara visualización de productos es una fortaleza. Podría incorporar más variedad visual, como iconos o banners, para mejorar la estética general y la diferenciación.</t>
+          <t>Las imágenes de productos son adecuadas; no obstante, implementar elementos visuales más dinámicos como vistas 360 grados o comparadores interactivos podría enriquecer la exploración. La adición de pequeños iconos relevantes a los encabezados de sección también sería beneficiosa.</t>
         </is>
       </c>
     </row>
@@ -514,13 +562,29 @@
           <t>Navigation &amp; UX</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ofrece una navegación intuitiva con filtros de categoría avanzados y una potente búsqueda, simplificando la compra en línea.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>La estructura de menú clara y los enlaces a artículos relacionados facilitan la exploración de su vasto repositorio de información tecnológica.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Se caracteriza por una organización de contenido lógica y un acceso sencillo a sus distintas secciones, garantizando una fluidez informativa.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>La barra de navegación es simple y muy visible, proporcionando acceso directo a secciones clave como 'Información' y 'Arma tu PC'. La barra de búsqueda también está bien situada.</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>La navegación directa es eficiente. Podría mejorar la UX con más opciones de filtrado o categorías secundarias para explorar componentes específicos.</t>
+          <t>La navegación actual es directa, pero la incorporación de un mega-menú más detallado podría soportar un crecimiento futuro en categorías de productos. Asegurar que todos los elementos interactivos ofrezcan retroalimentación visual clara mejoraría significativamente la confianza del usuario.</t>
         </is>
       </c>
     </row>
@@ -530,13 +594,29 @@
           <t>Organization &amp; Structure</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Organiza los productos en jerarquías lógicas, permitiendo a los usuarios una navegación sin esfuerzo hasta elementos específicos.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Estructura sus artículos con encabezados y párrafos bien definidos, lo que mejora la legibilidad de grandes volúmenes de texto técnico.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Emplea un formato de blog claro con categorías y etiquetas, ayudando eficazmente a los lectores a encontrar información relevante.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>La página de inicio separa eficazmente el eslogan principal de 'Componentes populares', creando un flujo de contenido limpio. Los enlaces de navegación principales están agrupados lógicamente en la parte superior derecha.</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>La organización por categorías populares es un buen comienzo. Se sugiere implementar una estructura de subcategorías más profunda para gestionar un catálogo más amplio.</t>
+          <t>Aunque el contenido está bien agrupado, la introducción de opciones de filtrado más avanzadas en las listas de productos permitiría una mayor personalización. Implementar 'migas de pan' (breadcrumbs) podría ofrecer a los usuarios un mejor contexto de su ubicación dentro de la jerarquía del sitio.</t>
         </is>
       </c>
     </row>
@@ -546,13 +626,29 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Cumple con estándares de accesibilidad, ofreciendo texto alternativo para imágenes y soporte para navegación con teclado.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Se esfuerza por mantener un contraste adecuado entre texto y fondo, mejorando la legibilidad para una amplia gama de usuarios.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Asegura que su contenido sea accesible con un diseño responsivo y compatibilidad con lectores de pantalla, beneficiando a todos.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>El diseño de alto contraste azul y blanco contribuye a una buena visibilidad general, y los elementos interactivos parecen tener un tamaño adecuado. Los tamaños de fuente son generalmente legibles.</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>El contraste es adecuado, lo que es un buen punto de partida. Sería beneficioso añadir mejoras para lectores de pantalla y opciones de tamaño de texto.</t>
+          <t>Mejorar el soporte de navegación por teclado y asegurar que todos los elementos interactivos estén correctamente etiquetados para lectores de pantalla es crucial. Ampliar las opciones de contraste de color o proporcionar un modo oscuro incrementaría aún más la usabilidad para individuos con discapacidades visuales.</t>
         </is>
       </c>
     </row>
@@ -562,13 +658,29 @@
           <t>Functionality</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dispone de una robusta plataforma de comercio electrónico con pasarelas de pago seguras y seguimiento exhaustivo de pedidos.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ofrece un rendimiento de carga veloz y funciones de búsqueda eficaces, permitiendo un acceso rápido a la información deseada.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Proporciona un sistema de comentarios totalmente funcional y botones para compartir en redes sociales, incentivando la interacción comunitaria.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>La barra de búsqueda es un elemento funcional clave, permitiendo a los usuarios encontrar componentes específicos con rapidez. Los enlaces de navegación también parecen ser completamente operativos y responsivos.</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>La funcionalidad de comparación es un valor distintivo. Podría expandir sus características para incluir un configurador de PC o filtros de productos avanzados.</t>
+          <t>Considerar la adición de un configurador de PC 'Arma tu PC', una función muy demandada en este sector, sería un gran avance. Un sistema de cuentas de usuario con historial de pedidos y listas de deseos también podría aumentar significativamente el compromiso.</t>
         </is>
       </c>
     </row>
@@ -578,13 +690,29 @@
           <t>Interactivity</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Permite a los usuarios dejar valoraciones y plantear preguntas sobre productos, creando así una comunidad de compradores activa.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Fomenta la participación mediante secciones de comentarios y encuestas, construyendo un diálogo continuo con su extensa audiencia.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ofrece campos de comentarios para discusiones y la opción de suscripción a boletines para mantenerse al día con las novedades.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Los enlaces de navegación existentes proporcionan interactividad básica, dirigiendo eficazmente a los usuarios a diferentes secciones. La barra de búsqueda ofrece retroalimentación inmediata al escribir.</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>El diseño limpio se enfoca en la información. Se recomienda integrar características interactivas como reseñas o un foro para enriquecer la experiencia del usuario.</t>
+          <t>Introducir herramientas de comparación de productos o cuestionarios interactivos para guiar a los usuarios en la elección de componentes sería valioso. Una sección de comentarios para artículos o páginas de productos podría fomentar el compromiso de la comunidad y el contenido generado por el usuario.</t>
         </is>
       </c>
     </row>
@@ -594,36 +722,68 @@
           <t>SEO</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Emplea descripciones de productos ricas en palabras clave y una estructura de URL amigable para los motores de búsqueda.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Optimiza sus artículos con meta descripciones, títulos pertinentes y enlaces internos, mejorando su visibilidad en línea.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Aplica prácticas SEO sólidas, incluyendo contenido de alta calidad y optimización de imágenes para el mejor posicionamiento.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Los títulos y encabezados parecen semánticamente relevantes para los componentes de PC, lo que sugiere una optimización básica de palabras clave. La estructura URL simple es propicia para la indexación.</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>La claridad de los nombres de productos ayuda. Debería centrarse en la creación de contenido relevante y una estructura de URL amigable para buscadores.</t>
+          <t>Optimizar las meta descripciones y etiquetas de título en todas las páginas para incluir más palabras clave relevantes y puntos de venta únicos. Desarrollar un blog con contenido valioso podría mejorar significativamente el tráfico orgánico y la autoridad del dominio.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Performance</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+          <t>Rendimiento Técnico</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Presenta tiempos de carga rápidos y una infraestructura robusta, soportando eficazmente un alto volumen de tráfico y transacciones.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Optimiza sus imágenes y scripts, lo que se traduce en una experiencia de navegación fluida y muy eficiente para el usuario.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Posee un sitio web ligero y bien codificado, asegurando una carga rápida incluso con una extensa cantidad de contenido multimedia.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>La página carga rápidamente según los elementos visibles, indicando un enfoque en la entrega eficiente de recursos. La responsividad sugiere un backend bien optimizado para operaciones básicas.</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>La simplicidad de su diseño contribuye a un buen rendimiento inicial. Mantener la optimización del rendimiento es vital a medida que el contenido crece.</t>
+          <t>Realizar auditorías de rendimiento regulares para identificar y resolver posibles cuellos de botella en la velocidad de carga de la página, especialmente con contenido dinámico. La optimización adicional del tamaño de las imágenes y el aprovechamiento del almacenamiento en caché del navegador podría conducir a una experiencia más consistentemente rápida.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Final Conclusion</t>
+          <t>Conclusión Final</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -632,7 +792,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RmCity ofrece una plataforma funcional y sencilla para explorar componentes de PC, destacando por su claridad visual y facilidad de navegación. Para competir mejor, se sugiere expandir las funcionalidades interactivas, profundizar la organización del contenido y enriquecer la experiencia del usuario con más herramientas de personalización y comunidad.</t>
+          <t>El sitio web presenta una base sólida con una interfaz limpia y una navegación intuitiva para los usuarios. Para mejorar su oferta, podría beneficiarse enormemente de la adición de funcionalidades avanzadas como un configurador de PC y herramientas de comparación. Optimizar el SEO con contenido de blog y descripciones meta más ricas, junto con una mayor interactividad y opciones de accesibilidad, potenciarían su relevancia y experiencia de usuario en el competitivo mercado de componentes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
conexion back con mi ia hecha (con ayuda de copilot y no se si funciona)
</commit_message>
<xml_diff>
--- a/IA/tablas_generadas/tablita.xlsx
+++ b/IA/tablas_generadas/tablita.xlsx
@@ -436,22 +436,22 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Tom's Hardware</t>
+          <t>(NamePage1)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>PC Gamer</t>
+          <t>(NamePage2)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>TechRadar</t>
+          <t>(NamePage3)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>PCity</t>
+          <t>(NamePage4)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -463,256 +463,256 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Typography &amp; Readability</t>
+          <t>Tipografía y legibilidad</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Estilo profesional. Utiliza fuentes sans-serif claras y tamaños legibles, optimizados para una lectura prolongada de análisis técnicos y guías detalladas.</t>
+          <t>El sitio emplea una tipografía sans-serif moderna para títulos y cuerpo. La jerarquía visual se establece mediante tamaños y pesos variados, asegurando una lectura fluida en sus extensos artículos y guías informativas.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Diseño dinámico. Emplea una combinación de tipografías atractivas para títulos y un cuerpo de texto nítido que facilita la inmersión en noticias y reseñas de juegos de PC.</t>
+          <t>Este portal utiliza una fuente clara y legible, priorizando el contraste en sus bloques de texto extensos. Los encabezados H1-H3 son distintivos, facilitando el escaneo rápido de las secciones principales del contenido editorial.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Apariencia moderna. Predominan tipografías limpias y bien espaciadas, asegurando una experiencia de lectura cómoda en todos sus artículos sobre tecnología y comparativas de hardware.</t>
+          <t>La plataforma presenta una tipografía estándar con excelente espaciado entre líneas y párrafos. La legibilidad general es alta, permitiendo a los usuarios absorber información técnica detallada sin fatiga visual innecesaria.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fuentes sencillas. La tipografía principal parece ser una sans-serif estándar que ofrece una legibilidad aceptable, aunque sin un estilo distintivo, lo que podría restarle impacto visual.</t>
+          <t>La interfaz usa una tipografía sans-serif que parece ser estándar y limpia. Los títulos principales son grandes y audaces, mientras que los textos de productos tienen un tamaño más pequeño con un contraste adecuado sobre fondo blanco.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PCity se beneficiaría de refinar su selección tipográfica, explorando fuentes modernas o variaciones de peso para crear una jerarquía visual más atractiva. Esto enriquecería la experiencia de lectura y le otorgaría un estilo distintivo.</t>
+          <t>Se sugiere explorar una familia tipográfica más distintiva que complemente la marca. Mantener la buena legibilidad de los títulos, pero revisar los tamaños del texto secundario para optimizar la comodidad visual en dispositivos variados.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Colors &amp; Branding</t>
+          <t>Colores y branding</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Identidad sobria. Su paleta de colores tiende a ser funcional, con tonos neutros y acentos para resaltar información clave, reforzando su imagen de autoridad técnica.</t>
+          <t>La paleta de colores del sitio combina tonos oscuros con acentos brillantes. La consistencia del logo y los elementos de marca se extiende a través de todo el sitio, reforzando su reconocimiento global y propuesta de valor tecnológico.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Marca vibrante. Combina colores oscuros con acentos brillantes, creando una estética que resuena con la cultura gamer y sus expectativas de contenido emocionante y visualmente atractivo.</t>
+          <t>Este portal exhibe una paleta de colores vibrantes, a menudo asociada con el gaming y la alta energía. El logo es prominente y se integra bien en un diseño que evoca pasión y dinamismo por el sector.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Esquema corporativo. Exhibe una paleta de colores equilibrada, a menudo con azules o verdes que transmiten confianza y modernidad, alineándose con su cobertura tecnológica.</t>
+          <t>La plataforma utiliza una combinación de azules y grises para transmitir seriedad y profesionalidad. El uso estratégico del logo refuerza la autoridad del medio en el ámbito técnico, proyectando una imagen de fiabilidad constante.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Esquema simple. El uso prominente de azul brillante en la cabecera con blanco para el contenido es funcional, pero carece de matices o un diseño de marca que lo distinga claramente.</t>
+          <t>El sitio presenta una cabecera azul brillante que contrasta fuertemente con un fondo blanco principal. El logo, un ratón con texto "Rity", es simple y se percibe como una imagen de marca básica y directa en su diseño general.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Es crucial que PCity desarrolle una paleta de colores más sofisticada y un diseño de logo que transmita una identidad de marca única. Dejar atrás la apariencia genérica le permitirá destacar en el mercado.</t>
+          <t>Considerar una paleta de colores más rica o matizada que el azul primario y el blanco. Desarrollar elementos visuales de marca consistentes que se extiendan más allá del logo para fortalecer la identidad y cohesión.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Visual Elements</t>
+          <t>Elementos visuales</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Imágenes técnicas. Presenta fotografías de alta calidad de componentes, gráficos detallados y capturas de pantalla que apoyan exhaustivamente sus análisis y comparativas.</t>
+          <t>El sitio integra fotografías de alta calidad, gráficos comparativos y videos explicativos. Los banners publicitarios son visibles pero no intrusivos, manteniendo el foco en el contenido editorial relevante y atractivo para el lector.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gráficos inmersivos. Incorpora abundantes imágenes de juegos, tráilers y videos que capturan la esencia del gaming, complementando sus reseñas y noticias de manera efectiva.</t>
+          <t>Este portal destaca por sus imágenes de juego inmersivas y capturas de pantalla de alta resolución en sus artículos. La iconografía es funcional, y las ilustraciones refuerzan la estética gamer, manteniendo la coherencia visual del medio.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Contenido multimedia. Utiliza un buen equilibrio de imágenes de productos, infografías y videos explicativos que enriquecen la comprensión de sus guías y análisis tecnológicos.</t>
+          <t>La plataforma emplea diagramas técnicos, tablas comparativas y fotos detalladas de componentes para ilustrar sus análisis. El diseño minimalista permite que las imágenes técnicas y los gráficos transmitan la información esencial de manera efectiva.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Componentes populares. Muestra imágenes cuadradas de productos sin un fondo coherente o estilo unificado, lo que las hace parecer básicas y no contribuye a una estética profesional.</t>
+          <t>Se observan imágenes de productos en formato de tarjeta, mostrando componentes de PC sobre fondos blancos uniformes. No se aprecian ilustraciones, iconografía diversa ni elementos visuales complejos más allá del logo y las fotografías de productos.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PCity podría estandarizar el estilo de sus imágenes de productos, quizás con fondos neutros o recortes uniformes. Integrar más elementos gráficos de apoyo visual a la información mejoraría la estética profesional.</t>
+          <t>Incorporar elementos visuales como ilustraciones o iconos para enriquecer la experiencia más allá de las fotografías de productos. Potenciar la sección de cabecera con un "hero" visual que capte la atención y comunique claramente el propósito del sitio.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Navigation &amp; UX</t>
+          <t>Navegación y UX</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Navegación profunda. Ofrece menús extensos y bien categorizados que permiten a los usuarios acceder rápidamente a diversas secciones, desde noticias hasta guías de compra especializadas.</t>
+          <t>El sitio ofrece un menú principal intuitivo con categorías claras y un buscador eficaz. Los breadcrumbs y los filtros avanzados mejoran la capacidad del usuario para explorar el contenido extenso y complejo con facilidad.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ruta clara. Su navegación es intuitiva, diseñada para que los aficionados a los videojuegos encuentren fácilmente noticias, reseñas y recursos específicos del ámbito gaming.</t>
+          <t>Este portal cuenta con una barra de navegación superior bien organizada y un buscador prominente. La estructura de menús facilita el acceso rápido a noticias, reseñas y guías, optimizando la experiencia de usuario general del visitante.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Interfaz amigable. Proporciona una experiencia de usuario fluida con menús claros y una estructura lógica, facilitando la exploración de sus amplias categorías de productos tecnológicos.</t>
+          <t>La plataforma presenta una navegación estructurada con menús desplegables y un robusto sistema de filtrado. La experiencia de usuario se beneficia de una jerarquía lógica que guía eficientemente por su vasto contenido técnico disponible.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Barra superior limitada. La navegación superior incluye 'Información', 'Arma tu PC' y 'Comparar', lo cual es funcional, pero carece de la profundidad necesaria para una experiencia completa.</t>
+          <t>La navegación superior es simple con enlaces ("Información", "Arma tu PC", "Comparar") y un buscador visible. No se aprecian breadcrumbs ni opciones de filtrado avanzadas en la vista principal, lo que simplifica la interacción inicial del usuario.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PCity debería expandir las opciones de navegación con menús desplegables y filtros, mejorando la usabilidad para que los usuarios encuentren componentes o información específica con mayor facilidad.</t>
+          <t>Implementar un sistema de breadcrumbs para mejorar la ubicación del usuario dentro del sitio, especialmente en secciones de productos o detalladas. Considerar la inclusión de filtros y categorías más específicas para la exploración eficiente de componentes.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Organization &amp; Structure</t>
+          <t>Organización y estructura</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Estructura modular. Presenta contenido en bloques bien definidos, con secciones dedicadas a noticias, reseñas, guías de compra y foros, facilitando la búsqueda de información técnica.</t>
+          <t>El contenido se organiza en un diseño de rejilla flexible, priorizando las noticias y reseñas más recientes. Las secciones están bien delimitadas, facilitando la comprensión y el acceso rápido a la información clave y actual.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Maquetación temática. Organiza su contenido por géneros de juegos, noticias recientes y reseñas destacadas, creando un flujo lógico que satisface los intereses de su audiencia gamer.</t>
+          <t>Este portal presenta una disposición de contenido dinámica, con énfasis en grandes bloques de noticias y análisis de juegos. La estructura fomenta la exploración de artículos relacionados, manteniendo el interés continuo del visitante.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Diseño por categorías. Estructura el sitio con secciones claras para diferentes tipos de tecnología y productos, permitiendo una exploración metódica de su vasto repositorio de información.</t>
+          <t>La plataforma adopta una disposición clara y estructurada, a menudo en columnas, para presentar sus análisis y guías. La priorización de contenidos se logra mediante encabezados y sumarios concisos en la página principal, orientando al usuario.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Disposición simple. El contenido se muestra en una columna central con un encabezado principal y una cuadrícula de productos, lo que resulta en una organización básica y un tanto monótona.</t>
+          <t>La estructura se observa con una cabecera, un título principal y una sección de "Componentes populares" en formato de rejilla. La disposición parece simple y directa, priorizando la visualización de los productos destacados en la página de inicio.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PCity se beneficiaría de una estructura de página más dinámica, utilizando columnas, secciones de contenido destacado y una jerarquía visual que guíe al usuario a través de la información relevante.</t>
+          <t>Es aconsejable introducir una jerarquía más marcada en la página de inicio, quizás con secciones dedicadas a noticias o guías. Mejorar la priorización de contenidos más allá de los productos populares para ofrecer una visión más completa y estructurada.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Accesibilidad</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cumplimiento técnico. Generalmente sigue buenas prácticas de accesibilidad web, asegurando que el contenido sea accesible para una audiencia diversa, incluyendo usuarios con discapacidades.</t>
+          <t>El sitio suele cumplir con estándares de accesibilidad, ofreciendo buen contraste y navegación por teclado eficiente. Las etiquetas ARIA y el texto alternativo en imágenes son comunes, mejorando la experiencia para todos los usuarios.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Diseño inclusivo. Busca optimizar la experiencia para todos los usuarios, prestando atención al contraste de colores y la navegación por teclado, mejorando la usabilidad general.</t>
+          <t>Este portal se esfuerza por la accesibilidad, con un contraste de color generalmente adecuado y foco visible en elementos interactivos. El texto alternativo en imágenes contribuye a una experiencia inclusiva para gamers diversos y con distintas necesidades.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Funcionalidad estándar. Implementa características de accesibilidad esenciales como texto alternativo y estructura semántica, facilitando la interacción con herramientas de asistencia.</t>
+          <t>La plataforma muestra un compromiso con la accesibilidad, utilizando buen contraste y permitiendo la navegación con teclado. El texto alternativo descriptivo en imágenes técnicas es un punto fuerte, ayudando a la comprensión general.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Potencial de mejora. Aunque el contraste de colores es adecuado, la ausencia de indicadores visuales o personalización sugiere oportunidades para una mayor inclusividad.</t>
+          <t>El contraste general del texto sobre fondos claros parece ser adecuado, aunque los enlaces de la cabecera sobre azul podrían ser optimizados. No se aprecia foco visible ni texto alternativo en la imagen, siendo aspectos importantes a revisar.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PCity necesita incorporar descripciones alternativas para imágenes y asegurar la navegación por teclado en todos los elementos interactivos. Ofrecer opciones de tamaño de texto también mejoraría significativamente la inclusividad.</t>
+          <t>Es crucial añadir texto alternativo descriptivo a todas las imágenes de productos y elementos gráficos para usuarios con discapacidad visual. Realizar pruebas de contraste para asegurar la legibilidad de todos los textos, especialmente los enlaces y el placeholder del buscador.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Functionality</t>
+          <t>Funcionalidad</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Herramientas robustas. Ofrece comparadores de productos, benchmarks interactivos y filtros avanzados, proporcionando una funcionalidad completa para el análisis de hardware.</t>
+          <t>El buscador avanzado del sitio, los filtros por categoría y los comparadores de productos son robustos y fiables. La estabilidad de sus componentes interactivos garantiza una experiencia fluida y confiable al usuario al explorar.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Características interactivas. Incluye filtros de búsqueda de juegos, secciones de comentarios activas y enlaces a tiendas, mejorando la experiencia del usuario y su interacción con el contenido.</t>
+          <t>Este portal ofrece un buscador eficaz y la posibilidad de filtrar contenidos por tipo o género de juego. La funcionalidad es sólida, permitiendo a los usuarios encontrar rápidamente análisis específicos o noticias relevantes del sector.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Utilidades prácticas. Provee buscadores eficientes, opciones de suscripción y una integración fluida de reseñas y guías de compra, asistiendo al usuario en su proceso de decisión.</t>
+          <t>La plataforma cuenta con herramientas de comparación detalladas y un sistema de búsqueda potente y preciso. La funcionalidad es excelente, proporcionando datos técnicos fiables y herramientas útiles para la toma de decisiones informadas.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Funciones básicas. La barra de búsqueda y los enlaces de navegación indican funcionalidades clave, pero la imagen no revela la profundidad de sus capacidades, pareciendo aún incipientes.</t>
+          <t>Se observa un campo de búsqueda funcional y enlaces para "Arma tu PC" y "Comparar", sugiriendo herramientas subyacentes. La visualización de productos en rejilla implica una funcionalidad básica de catálogo y exploración, aunque no se aprecian filtros en la vista.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PCity requiere expandir sus herramientas con filtros de producto más detallados y un comparador interactivo robusto. Integrar un configurador de PCs guiado ofrecería un valor añadido significativo a los usuarios.</t>
+          <t>Implementar filtros avanzados para la sección de productos, permitiendo a los usuarios refinar búsquedas por marca, tipo de componente o especificaciones. Asegurar que las herramientas "Arma tu PC" y "Comparar" sean intuitivas y robustas, ofreciendo una experiencia completa y útil.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Interactivity</t>
+          <t>Interactividad</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Compromiso profundo. Permite comentarios, foros de discusión y encuestas, fomentando una comunidad activa y el intercambio de conocimientos entre entusiastas del PC.</t>
+          <t>El sitio incorpora microinteracciones sutiles en botones y enlaces, proporcionando feedback visual instantáneo. Las animaciones son discretas, mejorando la experiencia sin distraer del contenido esencial y principal del portal.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Comunidad activa. Proporciona secciones de comentarios, integración de redes sociales y contenido generado por usuarios, cultivando una fuerte interacción entre su audiencia gamer.</t>
+          <t>Este portal presenta estados hover y focus bien definidos en sus elementos interactivos, lo cual es muy útil. Las animaciones se utilizan de forma estratégica para enriquecer la interfaz de usuario, especialmente en secciones multimedia o de noticias destacadas.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Participación guiada. Ofrece encuestas de satisfacción, comentarios en artículos y un sistema de valoración, animando a los usuarios a expresar sus opiniones y experiencias.</t>
+          <t>La plataforma ofrece interactividad clara con estados hover para enlaces y botones, mejorando la usabilidad general. Las transiciones son suaves y las microinteracciones son funcionales, apoyando la navegación precisa y eficiente del usuario.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Interacción limitada. La imagen no muestra elementos interactivos más allá de la navegación principal y los productos clickeables, lo que sugiere una falta de foros o personalización.</t>
+          <t>No se pueden observar directamente las microinteracciones ni los estados hover/focus desde la imagen estática. Se esperaría que los enlaces y la barra de búsqueda tuvieran algún tipo de feedback visual al interactuar, como cambios de color o subrayados.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Para fomentar el engagement, PCity podría añadir secciones de comentarios en los productos. Implementar un configurador de PCs interactivo y un sistema de votación para componentes aumentaría la participación del usuario.</t>
+          <t>Implementar estados hover y focus visualmente claros para todos los elementos interactivos, como enlaces de navegación y botones. Introducir microinteracciones sutiles para proporcionar feedback al usuario, mejorando la percepción de reactividad y dinamismo del sitio.</t>
         </is>
       </c>
     </row>
@@ -724,71 +724,75 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Autoridad establecida. Su antigüedad y contenido técnico de alta calidad le otorgan un fuerte posicionamiento en motores de búsqueda para términos relacionados con hardware y reviews.</t>
+          <t>El sitio optimiza sus títulos y meta descripciones, usando encabezados de forma lógica y datos estructurados. La buena arquitectura de enlaces internos y el rendimiento de carga contribuyen a su alta visibilidad en buscadores.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Optimización temática. Utiliza palabras clave relevantes para la industria del gaming, estructura de URLs amigable y enlaces internos, logrando una alta visibilidad en búsquedas de juegos y hardware.</t>
+          <t>Este portal utiliza meta descripciones atractivas y una estructura de encabezados coherente para el SEO. Los datos estructurados para reseñas y noticias, junto con un rápido tiempo de carga, favorecen su posicionamiento en Google.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Estrategia integral. Emplea una sólida arquitectura de enlaces, contenido optimizado para palabras clave y una rápida velocidad de carga, asegurando una fuerte presencia en resultados de búsqueda.</t>
+          <t>La plataforma implementa títulos y meta descripciones precisas, con uso adecuado de canonicals y robots.txt. Su rendimiento es sólido, y la organización del contenido con encabezados beneficia directamente su clasificación SEO orgánica.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ausencia de evidencia. La información visual no permite inferir su estrategia SEO; sin embargo, necesitaría una optimización cuidadosa de títulos, descripciones y estructura de contenido para competir.</t>
+          <t>Se observan títulos principales y subtítulos (H1-H2) con texto relevante, lo que es positivo para el SEO. Sin embargo, no se pueden inferir meta descripciones, datos estructurados o un rendimiento de carga desde la captura de pantalla estática.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PCity debe implementar una estrategia SEO robusta que incluya investigación de palabras clave, optimización de metadatos y una estructura de enlaces interna fuerte. Esto es crucial para su visibilidad y para competir eficazmente.</t>
+          <t>Revisar y optimizar los meta títulos y descripciones para cada página, incluyendo palabras clave relevantes del sector. Considerar la implementación de datos estructurados para los productos y las herramientas de comparación, mejorando la visibilidad en resultados enriquecidos.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Content Freshness</t>
+          <t>Coherencia de diseño</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Contenido actualizado. Publica diariamente noticias, reseñas de hardware recién lanzado y guías actualizadas, manteniendo a su audiencia informada sobre las últimas tendencias.</t>
+          <t>El sitio mantiene una coherencia de diseño notable a través de su tipografía, paleta de colores y estilo gráfico general. La uniformidad visual en sus diferentes secciones refuerza la identidad de marca, generando confianza en los usuarios.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Flujo constante. Ofrece una corriente continua de noticias de juegos, parches, eventos y reseñas de nuevos lanzamientos, manteniendo su contenido pertinente y atractivo para gamers.</t>
+          <t>Este portal exhibe una fuerte coherencia de diseño, donde los elementos visuales y el estilo se alinean con su público objetivo. La uniformidad en la presentación de contenido y branding crea una experiencia inmersiva y muy atractiva.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Publicación regular. Actualiza frecuentemente sus artículos con las últimas novedades tecnológicas, cubriendo lanzamientos de productos y tendencias de la industria para mantener la relevancia.</t>
+          <t>La plataforma demuestra una alta coherencia de diseño en su estructura, uso de colores y elementos tipográficos clave. Esta uniformidad contribuye a una experiencia de usuario predecible y profesional a lo largo de todo el sitio.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Frecuencia incierta. La imagen no permite determinar la regularidad de las actualizaciones de contenido o la frecuencia de adición de nuevos productos, crucial para la relevancia.</t>
+          <t>La cabecera, los títulos y las tarjetas de productos muestran una coherencia básica en su estilo visual. La simplicidad del diseño, aunque funcional, carece de elementos unificadores que aporten una estética más elaborada y distintiva al conjunto.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PCity debería asegurar una actualización constante de productos y contenido informativo, publicando artículos sobre nuevas tecnologías y lanzamientos. Esto mantendría el interés del usuario y su relevancia en el sector.</t>
+          <t>Desarrollar una guía de estilos clara para asegurar que todos los componentes visuales futuros mantengan la misma línea estética. Incorporar patrones de diseño consistentes para los elementos interactivos y los módulos de contenido, elevando la profesionalidad.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Conclusión final</t>
+        </is>
+      </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PCity muestra una base sólida para la comparación y configuración de PCs. Para maximizar su potencial, debe enriquecer su diseño visual y tipográfico, expandir la profundidad de su navegación y funcionalidades interactivas, e implementar una estrategia SEO y de contenido fresco para atraer y retener usuarios de manera efectiva.</t>
+          <t>Para Website4, las mejoras prioritarias incluyen enriquecer la paleta de colores y elementos visuales con un "hero" distintivo en la cabecera. Es crucial implementar texto alternativo y asegurar el contraste para la accesibilidad, además de añadir filtros avanzados para productos y robustecer las herramientas de "Arma tu PC" y "Comparar". Finalmente, optimizar el SEO con metadatos estructurados y mejorar la interactividad con estados visuales claros elevará significativamente la experiencia de usuario y la visibilidad del portal.</t>
         </is>
       </c>
     </row>

</xml_diff>